<commit_message>
data: update werkstätten 2026-03-16
</commit_message>
<xml_diff>
--- a/data/werkstaetten.xlsx
+++ b/data/werkstaetten.xlsx
@@ -9638,7 +9638,7 @@
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
-        <v>6442</v>
+        <v>6441</v>
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
@@ -9647,22 +9647,22 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>SVS Wolfurt</t>
+          <t>SVS Wörgl</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Senderstraße 8b</t>
+          <t>Ferdinand Raimundstraße 15</t>
         </is>
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>6960</t>
+          <t>6300</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>Wolfurt-Bahnhof</t>
+          <t>Wörgl</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -9683,20 +9683,20 @@
         </is>
       </c>
       <c r="L165" s="2" t="n">
-        <v>47.4567143</v>
+        <v>47.4931471</v>
       </c>
       <c r="M165" s="2" t="n">
-        <v>9.739088600000001</v>
+        <v>12.060234</v>
       </c>
       <c r="N165" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6442-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6441-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
-        <v>6443</v>
+        <v>6442</v>
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
@@ -9705,22 +9705,22 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>SVS Wolfsberg</t>
+          <t>SVS Wolfurt</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>Kirchbichelstraße 1</t>
+          <t>Senderstraße 8b</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>9400</t>
+          <t>6960</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>Wolfsberg, Kärnten</t>
+          <t>Wolfurt-Bahnhof</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -9735,22 +9735,26 @@
       </c>
       <c r="I166" s="2" t="inlineStr"/>
       <c r="J166" s="2" t="inlineStr"/>
-      <c r="K166" s="3" t="inlineStr"/>
+      <c r="K166" s="3" t="inlineStr">
+        <is>
+          <t>http://www.oebb.at/ts</t>
+        </is>
+      </c>
       <c r="L166" s="2" t="n">
-        <v>46.839886</v>
+        <v>47.4567143</v>
       </c>
       <c r="M166" s="2" t="n">
-        <v>14.8374699</v>
+        <v>9.739088600000001</v>
       </c>
       <c r="N166" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6443-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6442-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
-        <v>6444</v>
+        <v>6443</v>
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
@@ -9759,22 +9763,22 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>SVS Wr. Neustadt</t>
+          <t>SVS Wolfsberg</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Neunkirchnerstraße 82</t>
+          <t>Kirchbichelstraße 1</t>
         </is>
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>2700</t>
+          <t>9400</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>Wiener Neustadt</t>
+          <t>Wolfsberg, Kärnten</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -9789,26 +9793,22 @@
       </c>
       <c r="I167" s="2" t="inlineStr"/>
       <c r="J167" s="2" t="inlineStr"/>
-      <c r="K167" s="3" t="inlineStr">
-        <is>
-          <t>http://www.oebb.at/ts</t>
-        </is>
-      </c>
+      <c r="K167" s="3" t="inlineStr"/>
       <c r="L167" s="2" t="n">
-        <v>47.8093458</v>
+        <v>46.839886</v>
       </c>
       <c r="M167" s="2" t="n">
-        <v>16.234883</v>
+        <v>14.8374699</v>
       </c>
       <c r="N167" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6444-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6443-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
-        <v>6446</v>
+        <v>6444</v>
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
@@ -9817,22 +9817,22 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Geschäftsfeld Güterwagen, Werk Jedlersdorf</t>
+          <t>SVS Wr. Neustadt</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Winkeläckerweg 1</t>
+          <t>Neunkirchnerstraße 82</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>1210</t>
+          <t>2700</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>Wien</t>
+          <t>Wiener Neustadt</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -9847,18 +9847,26 @@
       </c>
       <c r="I168" s="2" t="inlineStr"/>
       <c r="J168" s="2" t="inlineStr"/>
-      <c r="K168" s="3" t="inlineStr"/>
-      <c r="L168" s="2" t="inlineStr"/>
-      <c r="M168" s="2" t="inlineStr"/>
+      <c r="K168" s="3" t="inlineStr">
+        <is>
+          <t>http://www.oebb.at/ts</t>
+        </is>
+      </c>
+      <c r="L168" s="2" t="n">
+        <v>47.8093458</v>
+      </c>
+      <c r="M168" s="2" t="n">
+        <v>16.234883</v>
+      </c>
       <c r="N168" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6446-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6444-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
-        <v>6447</v>
+        <v>6446</v>
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
@@ -9867,17 +9875,17 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>SVS Wien FJB</t>
+          <t>Geschäftsfeld Güterwagen, Werk Jedlersdorf</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>Spittelauerlände 33</t>
+          <t>Winkeläckerweg 1</t>
         </is>
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>1090</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
@@ -9897,26 +9905,18 @@
       </c>
       <c r="I169" s="2" t="inlineStr"/>
       <c r="J169" s="2" t="inlineStr"/>
-      <c r="K169" s="3" t="inlineStr">
-        <is>
-          <t>http://www.oebb.at/ts</t>
-        </is>
-      </c>
-      <c r="L169" s="2" t="n">
-        <v>48.2253633</v>
-      </c>
-      <c r="M169" s="2" t="n">
-        <v>16.3561956</v>
-      </c>
+      <c r="K169" s="3" t="inlineStr"/>
+      <c r="L169" s="2" t="inlineStr"/>
+      <c r="M169" s="2" t="inlineStr"/>
       <c r="N169" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6447-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6446-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
-        <v>6448</v>
+        <v>6447</v>
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
@@ -9925,17 +9925,17 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>SVS Wien Kledering</t>
+          <t>SVS Wien FJB</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>Ruthnergasse 2a</t>
+          <t>Spittelauerlände 33</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>1210</t>
+          <t>1090</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -9961,20 +9961,20 @@
         </is>
       </c>
       <c r="L170" s="2" t="n">
-        <v>48.2662711</v>
+        <v>48.2253633</v>
       </c>
       <c r="M170" s="2" t="n">
-        <v>16.4083928</v>
+        <v>16.3561956</v>
       </c>
       <c r="N170" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6448-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6447-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
-        <v>6449</v>
+        <v>6448</v>
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
@@ -9983,17 +9983,17 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>SVS Wien Matzleinsdorf</t>
+          <t>SVS Wien Kledering</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>Margaretengürtel 35</t>
+          <t>Ruthnergasse 2a</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>1100</t>
+          <t>1210</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -10019,20 +10019,20 @@
         </is>
       </c>
       <c r="L171" s="2" t="n">
-        <v>48.1794494</v>
+        <v>48.2662711</v>
       </c>
       <c r="M171" s="2" t="n">
-        <v>16.354983</v>
+        <v>16.4083928</v>
       </c>
       <c r="N171" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6449-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6448-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
-        <v>6450</v>
+        <v>6449</v>
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
@@ -10041,17 +10041,17 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>Werk Wien Simmering</t>
+          <t>SVS Wien Matzleinsdorf</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>Grillgasse 48</t>
+          <t>Margaretengürtel 35</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>1410</t>
+          <t>1100</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -10077,20 +10077,20 @@
         </is>
       </c>
       <c r="L172" s="2" t="n">
-        <v>48.168779</v>
+        <v>48.1794494</v>
       </c>
       <c r="M172" s="2" t="n">
-        <v>16.4088199</v>
+        <v>16.354983</v>
       </c>
       <c r="N172" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6450-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6449-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
-        <v>6451</v>
+        <v>6450</v>
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
@@ -10099,17 +10099,17 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>SVS Wien West</t>
+          <t>Werk Wien Simmering</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>Avediktstraße 2</t>
+          <t>Grillgasse 48</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>1150</t>
+          <t>1410</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
@@ -10135,20 +10135,20 @@
         </is>
       </c>
       <c r="L173" s="2" t="n">
-        <v>48.1943829</v>
+        <v>48.168779</v>
       </c>
       <c r="M173" s="2" t="n">
-        <v>16.3235143</v>
+        <v>16.4088199</v>
       </c>
       <c r="N173" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6451-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6450-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
-        <v>6452</v>
+        <v>6451</v>
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
@@ -10157,22 +10157,22 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>SVS Wels</t>
+          <t>SVS Wien West</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>Flugplatzstraße 12a</t>
+          <t>Avediktstraße 2</t>
         </is>
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>4600</t>
+          <t>1150</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>Wels</t>
+          <t>Wien</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -10193,20 +10193,20 @@
         </is>
       </c>
       <c r="L174" s="2" t="n">
-        <v>48.1770433</v>
+        <v>48.1943829</v>
       </c>
       <c r="M174" s="2" t="n">
-        <v>14.0471108</v>
+        <v>16.3235143</v>
       </c>
       <c r="N174" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6452-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6451-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
-        <v>6453</v>
+        <v>6452</v>
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
@@ -10215,22 +10215,22 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>SVS Waidhofen/Ybbs</t>
+          <t>SVS Wels</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>Wiener Straße 45b</t>
+          <t>Flugplatzstraße 12a</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>3340</t>
+          <t>4600</t>
         </is>
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>Waidhofen/Ybbs</t>
+          <t>Wels</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -10251,20 +10251,20 @@
         </is>
       </c>
       <c r="L175" s="2" t="n">
-        <v>47.9701775</v>
+        <v>48.1770433</v>
       </c>
       <c r="M175" s="2" t="n">
-        <v>14.7638161</v>
+        <v>14.0471108</v>
       </c>
       <c r="N175" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6453-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6452-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
-        <v>6454</v>
+        <v>6453</v>
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
@@ -10273,22 +10273,22 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>SVS Villach</t>
+          <t>SVS Waidhofen/Ybbs</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>Heizhausstraße 49</t>
+          <t>Wiener Straße 45b</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>9500</t>
+          <t>3340</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>Villach</t>
+          <t>Waidhofen/Ybbs</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -10309,20 +10309,20 @@
         </is>
       </c>
       <c r="L176" s="2" t="n">
-        <v>46.6025529</v>
+        <v>47.9701775</v>
       </c>
       <c r="M176" s="2" t="n">
-        <v>13.8367749</v>
+        <v>14.7638161</v>
       </c>
       <c r="N176" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6454-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6453-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
-        <v>6455</v>
+        <v>6454</v>
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
@@ -10331,22 +10331,22 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>SVS St. Pölten</t>
+          <t>SVS Villach</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Werkstättenstraße  17</t>
+          <t>Heizhausstraße 49</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>3100</t>
+          <t>9500</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>St. Pölten</t>
+          <t>Villach</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -10367,20 +10367,20 @@
         </is>
       </c>
       <c r="L177" s="2" t="n">
-        <v>48.1929083</v>
+        <v>46.6025529</v>
       </c>
       <c r="M177" s="2" t="n">
-        <v>15.6122777</v>
+        <v>13.8367749</v>
       </c>
       <c r="N177" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6455-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6454-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
-        <v>6456</v>
+        <v>6455</v>
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
@@ -10389,22 +10389,22 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>SVS Salzburg</t>
+          <t>SVS St. Pölten</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>Röcklbrunnerstraße 12</t>
+          <t>Werkstättenstraße  17</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>5020</t>
+          <t>3100</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>Salzburg</t>
+          <t>St. Pölten</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -10425,20 +10425,20 @@
         </is>
       </c>
       <c r="L178" s="2" t="n">
-        <v>47.8051393</v>
+        <v>48.1929083</v>
       </c>
       <c r="M178" s="2" t="n">
-        <v>13.0380686</v>
+        <v>15.6122777</v>
       </c>
       <c r="N178" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6456-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6455-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
-        <v>6457</v>
+        <v>6456</v>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
@@ -10447,22 +10447,22 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Werk Linz</t>
+          <t>SVS Salzburg</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>Unionstraße 24</t>
+          <t>Röcklbrunnerstraße 12</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>5020</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>Linz</t>
+          <t>Salzburg</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -10482,17 +10482,21 @@
           <t>http://www.oebb.at/ts</t>
         </is>
       </c>
-      <c r="L179" s="2" t="inlineStr"/>
-      <c r="M179" s="2" t="inlineStr"/>
+      <c r="L179" s="2" t="n">
+        <v>47.8051393</v>
+      </c>
+      <c r="M179" s="2" t="n">
+        <v>13.0380686</v>
+      </c>
       <c r="N179" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6457-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6456-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
-        <v>6458</v>
+        <v>6457</v>
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
@@ -10501,22 +10505,22 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>SVS Krems</t>
+          <t>Werk Linz</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Am Frachtenbahnhof 5</t>
+          <t>Unionstraße 24</t>
         </is>
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>3500</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>Krems an der Donau</t>
+          <t>Linz</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -10536,21 +10540,17 @@
           <t>http://www.oebb.at/ts</t>
         </is>
       </c>
-      <c r="L180" s="2" t="n">
-        <v>48.4073591</v>
-      </c>
-      <c r="M180" s="2" t="n">
-        <v>15.6047696</v>
-      </c>
+      <c r="L180" s="2" t="inlineStr"/>
+      <c r="M180" s="2" t="inlineStr"/>
       <c r="N180" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6458-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6457-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
-        <v>6459</v>
+        <v>6458</v>
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
@@ -10559,22 +10559,22 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Werk Knittelfeld - Radsätze</t>
+          <t>SVS Krems</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>Lobmingerstraße 1</t>
+          <t>Am Frachtenbahnhof 5</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>8720</t>
+          <t>3500</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>Knittelfeld</t>
+          <t>Krems an der Donau</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -10595,20 +10595,20 @@
         </is>
       </c>
       <c r="L181" s="2" t="n">
-        <v>47.2111722</v>
+        <v>48.4073591</v>
       </c>
       <c r="M181" s="2" t="n">
-        <v>14.8317274</v>
+        <v>15.6047696</v>
       </c>
       <c r="N181" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6459-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6458-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
-        <v>6460</v>
+        <v>6459</v>
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
@@ -10617,22 +10617,22 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>SVS Kledering</t>
+          <t>Werk Knittelfeld - Radsätze</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>Ostbahnstraße 1</t>
+          <t>Lobmingerstraße 1</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8720</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>Kledering</t>
+          <t>Knittelfeld</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -10653,20 +10653,20 @@
         </is>
       </c>
       <c r="L182" s="2" t="n">
-        <v>48.1348684</v>
+        <v>47.2111722</v>
       </c>
       <c r="M182" s="2" t="n">
-        <v>16.4411144</v>
+        <v>14.8317274</v>
       </c>
       <c r="N182" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6460-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6459-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="n">
-        <v>6461</v>
+        <v>6460</v>
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
@@ -10675,22 +10675,22 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>SVS Innsbruck</t>
+          <t>SVS Kledering</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>Wiltenberg 1a</t>
+          <t>Ostbahnstraße 1</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>6020</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>Innsbruck</t>
+          <t>Kledering</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -10711,20 +10711,20 @@
         </is>
       </c>
       <c r="L183" s="2" t="n">
-        <v>47.2538984</v>
+        <v>48.1348684</v>
       </c>
       <c r="M183" s="2" t="n">
-        <v>11.3815033</v>
+        <v>16.4411144</v>
       </c>
       <c r="N183" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6461-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6460-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
-        <v>6462</v>
+        <v>6461</v>
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
@@ -10733,22 +10733,22 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>SVS Graz</t>
+          <t>SVS Innsbruck</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>Bahnhofgürtel 40</t>
+          <t>Wiltenberg 1a</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>8020</t>
+          <t>6020</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>Graz</t>
+          <t>Innsbruck</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -10769,14 +10769,14 @@
         </is>
       </c>
       <c r="L184" s="2" t="n">
-        <v>47.0799482</v>
+        <v>47.2538984</v>
       </c>
       <c r="M184" s="2" t="n">
-        <v>15.4148748</v>
+        <v>11.3815033</v>
       </c>
       <c r="N184" s="3" t="inlineStr">
         <is>
-          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6462-oebb-technische-services-gmbh.html</t>
+          <t>http://www.werkstattatlas.info/unternehmen/werkstaetten/6461-oebb-technische-services-gmbh.html</t>
         </is>
       </c>
     </row>

</xml_diff>